<commit_message>
removed accidentally commented code and added auropharma
</commit_message>
<xml_diff>
--- a/ltp prev.xlsx
+++ b/ltp prev.xlsx
@@ -10,7 +10,7 @@
     <sheet name="30" sheetId="1" r:id="rId1"/>
     <sheet name="15" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="144525"/>
 </workbook>
 </file>
 
@@ -940,7 +940,9 @@
       <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="2"/>
+      <c r="B2" s="2">
+        <v>5188.3999999999996</v>
+      </c>
       <c r="C2" s="1"/>
       <c r="F2" s="2"/>
     </row>
@@ -948,7 +950,9 @@
       <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="2"/>
+      <c r="B3" s="2">
+        <v>2288.6999999999998</v>
+      </c>
       <c r="C3" s="1"/>
       <c r="F3" s="2"/>
     </row>
@@ -956,14 +960,18 @@
       <c r="A4" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="2"/>
+      <c r="B4" s="2">
+        <v>7736</v>
+      </c>
       <c r="F4" s="2"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="2"/>
+      <c r="B5" s="2">
+        <v>1966.1</v>
+      </c>
       <c r="C5" s="1"/>
       <c r="F5" s="2"/>
     </row>
@@ -971,7 +979,9 @@
       <c r="A6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="2"/>
+      <c r="B6" s="2">
+        <v>896.3</v>
+      </c>
       <c r="C6" s="1"/>
       <c r="F6" s="2"/>
     </row>
@@ -979,35 +989,45 @@
       <c r="A7" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="2"/>
+      <c r="B7" s="2">
+        <v>216.97</v>
+      </c>
       <c r="F7" s="2"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>39</v>
       </c>
-      <c r="B8" s="2"/>
+      <c r="B8" s="2">
+        <v>377.05</v>
+      </c>
       <c r="F8" s="2"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="2"/>
+      <c r="B9" s="2">
+        <v>569.75</v>
+      </c>
       <c r="F9" s="2"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>40</v>
       </c>
-      <c r="B10" s="2"/>
+      <c r="B10" s="2">
+        <v>1731.8</v>
+      </c>
       <c r="F10" s="2"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="2"/>
+      <c r="B11" s="2">
+        <v>17759</v>
+      </c>
       <c r="C11" s="1"/>
       <c r="F11" s="2"/>
     </row>
@@ -1015,14 +1035,18 @@
       <c r="A12" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="2"/>
+      <c r="B12" s="2">
+        <v>764.4</v>
+      </c>
       <c r="F12" s="2"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>41</v>
       </c>
-      <c r="B13" s="2"/>
+      <c r="B13" s="2">
+        <v>2004.4</v>
+      </c>
       <c r="C13" s="1"/>
       <c r="F13" s="2"/>
     </row>
@@ -1030,7 +1054,9 @@
       <c r="A14" t="s">
         <v>42</v>
       </c>
-      <c r="B14" s="2"/>
+      <c r="B14" s="2">
+        <v>4451</v>
+      </c>
       <c r="C14" s="1"/>
       <c r="F14" s="2"/>
     </row>
@@ -1038,14 +1064,18 @@
       <c r="A15" t="s">
         <v>43</v>
       </c>
-      <c r="B15" s="2"/>
+      <c r="B15" s="2">
+        <v>874.7</v>
+      </c>
       <c r="F15" s="2"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>44</v>
       </c>
-      <c r="B16" s="2"/>
+      <c r="B16" s="2">
+        <v>7707.5</v>
+      </c>
       <c r="C16" s="1"/>
       <c r="F16" s="2"/>
     </row>
@@ -1053,14 +1083,18 @@
       <c r="A17" t="s">
         <v>28</v>
       </c>
-      <c r="B17" s="2"/>
+      <c r="B17" s="2">
+        <v>24813.1</v>
+      </c>
       <c r="F17" s="2"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>32</v>
       </c>
-      <c r="B18" s="2"/>
+      <c r="B18" s="2">
+        <v>1372.6</v>
+      </c>
       <c r="C18" s="1"/>
       <c r="F18" s="2"/>
     </row>
@@ -1068,7 +1102,9 @@
       <c r="A19" t="s">
         <v>35</v>
       </c>
-      <c r="B19" s="2"/>
+      <c r="B19" s="2">
+        <v>692.05</v>
+      </c>
       <c r="F19" s="2"/>
     </row>
   </sheetData>

</xml_diff>